<commit_message>
Build competition-ready Truecell review workspace
</commit_message>
<xml_diff>
--- a/outputs/A_invoice_register.xlsx
+++ b/outputs/A_invoice_register.xlsx
@@ -23,7 +23,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Validation Report'!$A$1:$H$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Page Audit'!$A$1:$L$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Provenance'!$A$1:$E$49</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Read me'!$A$1:$B$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Read me'!$A$1:$B$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Cell Evidence'!$A$1:$M$613</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Verification'!$A$1:$B$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Constraints'!$A$1:$H$2</definedName>
@@ -3817,7 +3817,7 @@
         <v>0.98</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.126</v>
+        <v>0.19</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
@@ -3859,7 +3859,7 @@
         <v>0.98</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0.119</v>
+        <v>0.179</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -3901,7 +3901,7 @@
         <v>0.98</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.129</v>
+        <v>0.159</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -4994,7 +4994,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5032,95 +5032,131 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>0.781</v>
-      </c>
-    </row>
-    <row r="4" ht="34" customHeight="1">
+        <v>1.081</v>
+      </c>
+    </row>
+    <row r="4" ht="119" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Yellow cells</t>
+          <t>Text encoding</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Review required. See Validation Report for the reason and source row.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="34" customHeight="1">
+          <t>All XLSX string fields use a reversible encoding: a literal backslash is doubled; XML-forbidden code points use a backslash followed by u and four hexadecimal digits. An underscore starting an OOXML escape-like sequence uses the same Unicode encoding. Decode left to right, treating each doubled backslash as one literal backslash. The full audit JSON and saved workspace retain the original strings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="68" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Source row</t>
+          <t>Long text</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Data row within the extracted source table, excluding detected headers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="34" customHeight="1">
+          <t>Values exceeding Excel's 32767-character cell limit show an explicit preview. The Long Text sheet preserves the complete encoded value in numbered chunks. Join its chunks in order before decoding the text encoding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="68" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Confidence</t>
+          <t>Small numbers</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Extraction heuristic / OCR score, not a calibrated probability of correctness.</t>
+          <t>Numbers below Excel's normal floating-point range remain exact text. Numbers needing more than 12 decimal places use General formatting; percentages needing more than 12 display decimals remain text, avoiding a false zero.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Dates</t>
+          <t>Yellow cells</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>ISO and unambiguous day-first dates are typed. Ambiguous dates stay text.</t>
+          <t>Review required. See Validation Report for the reason and source row.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Source row</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Source strings are stored as text. No source formulas are executed.</t>
+          <t>Data row within the extracted source table, excluding detected headers.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Cell evidence</t>
+          <t>Confidence</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Ctrl+click a linked data cell for its source bounding box and original readings.</t>
+          <t>Extraction heuristic / OCR score, not a calibrated probability of correctness.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>Dates</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>ISO and unambiguous day-first dates are typed. Ambiguous dates stay text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Source strings are stored as text. No source formulas are executed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Cell evidence</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Ctrl+click a linked data cell for its source bounding box and original readings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
           <t>Repair proposals</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Arithmetic-derived suggestions only. Source documents may contain errors. Never applied automatically.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B10"/>
+  <autoFilter ref="A1:B13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -32807,7 +32843,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>78fab1cd80c4d6ee6896332db7bd3fe025e9233b93f58657cffd17e47558a5aa</t>
+          <t>0adb9c9f6ed1d48018e7fb748ca49af5acb12e5b693d9d9f091d0de5c8c68532</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add auditable multipage review workflow
</commit_message>
<xml_diff>
--- a/outputs/A_invoice_register.xlsx
+++ b/outputs/A_invoice_register.xlsx
@@ -10,25 +10,27 @@
     <sheet name="Data 1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Validation Report" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Page Audit" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Provenance" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Read me" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Cell Evidence" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Verification" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Constraints" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Repair Proposals" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Correction History" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Join Receipt" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Provenance" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Read me" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Cell Evidence" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Verification" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Constraints" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Repair Proposals" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Correction History" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data 1'!$A$1:$L$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Validation Report'!$A$1:$H$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Page Audit'!$A$1:$L$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Provenance'!$A$1:$E$49</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Read me'!$A$1:$B$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Cell Evidence'!$A$1:$M$613</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Verification'!$A$1:$B$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Constraints'!$A$1:$H$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Repair Proposals'!$A$1:$I$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Correction History'!$A$1:$I$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Join Receipt'!$A$1:$H$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Provenance'!$A$1:$E$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Read me'!$A$1:$B$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Cell Evidence'!$A$1:$M$613</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Verification'!$A$1:$B$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Constraints'!$A$1:$H$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Repair Proposals'!$A$1:$I$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Correction History'!$A$1:$I$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3562,6 +3564,79 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Excel row</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Observed</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Supporting equations</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Caution</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
@@ -3817,7 +3892,7 @@
         <v>0.98</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.19</v>
+        <v>0.277</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
@@ -3859,7 +3934,7 @@
         <v>0.98</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0.179</v>
+        <v>0.9419999999999999</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -3901,7 +3976,7 @@
         <v>0.98</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.159</v>
+        <v>0.999</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -3932,6 +4007,163 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Data sheet</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Source pages</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Page joins</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Repeated headers removed</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Split rows recovered</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>PDF page</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Source rows on page</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Output rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="17" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Data 1</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3" ht="17" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Data 1</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" ht="17" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Data 1</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H4"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4988,7 +5220,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5032,7 +5264,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>1.081</v>
+        <v>5.02</v>
       </c>
     </row>
     <row r="4" ht="119" customHeight="1">
@@ -5161,7 +5393,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -32798,7 +33030,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -32843,7 +33075,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>0adb9c9f6ed1d48018e7fb748ca49af5acb12e5b693d9d9f091d0de5c8c68532</t>
+          <t>e76cf6edfde5fdda07ef551118ed7c18fa19beeb759ac1a74c57eaad5a478f16</t>
         </is>
       </c>
     </row>
@@ -32945,7 +33177,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -33042,77 +33274,4 @@
   <autoFilter ref="A1:H2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Table</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Excel row</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Column</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Observed</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Supporting equations</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Evidence</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Caution</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:I1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>